<commit_message>
Lägg till lösenord i Excel
</commit_message>
<xml_diff>
--- a/Allsvenskan_Tipstävling_2026.xlsx
+++ b/Allsvenskan_Tipstävling_2026.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Privat\Hemsida\Verktyg\Tipstävling Allsvenskan 2026 - kopia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Privat\Hemsida\Verktyg\Tipstävling Allsvenskan 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B95BF5BD-ECEB-4FD7-8AFE-47DB55C5DB9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4117C49B-D6A3-4480-B5A1-2DA674B34825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="19440" windowHeight="10440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2085,6 +2085,7 @@
       <c r="Q18" s="4"/>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="6MZ69Mb0Q0VnY9JI8AQUO37Uz2NSi7kaCFkWHMir3t5SxS/0GVJSiOZZl+HDnBHVcH40nv8BO4oFWNIpy6SZWg==" saltValue="wRyeDbZXx3jdirxZSpBcsw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <conditionalFormatting sqref="L2:P17">
     <cfRule type="colorScale" priority="1">
       <colorScale>

</xml_diff>